<commit_message>
added my notes and updated the kpi tracker based on feedback provided
</commit_message>
<xml_diff>
--- a/submissions/excel/excel_06b_kpis_tracker.xlsx
+++ b/submissions/excel/excel_06b_kpis_tracker.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\venti\Downloads\training\excel\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\venti\Downloads\idynamics-training\idynamics-analyst-training\submissions\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{E6F16AFC-3B76-40C4-863C-27B3E4BA5757}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A5B71485-FDB5-43BB-9286-EE88DB23DF77}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" firstSheet="1" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1348,7 +1348,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1461" uniqueCount="655">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1462" uniqueCount="656">
   <si>
     <t>HISTORICAL BASELINE — 2024 &amp; 2025 ACTUALS</t>
   </si>
@@ -3313,6 +3313,9 @@
   </si>
   <si>
     <t xml:space="preserve">Excel 02 </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> - Contraction MRR</t>
   </si>
 </sst>
 </file>
@@ -3867,12 +3870,6 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="33" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="29" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="26" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="34" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="13" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="35" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -3899,6 +3896,12 @@
     <xf numFmtId="0" fontId="36" fillId="13" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="29" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="26" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Currency" xfId="1" builtinId="4"/>
@@ -3906,18 +3909,6 @@
     <cellStyle name="Percent" xfId="2" builtinId="5"/>
   </cellStyles>
   <dxfs count="21">
-    <dxf>
-      <numFmt numFmtId="175" formatCode="&quot;$&quot;#,##0.00"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="175" formatCode="&quot;$&quot;#,##0.00"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="175" formatCode="&quot;$&quot;#,##0.00"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="22" formatCode="mmm/yy"/>
-    </dxf>
     <dxf>
       <font>
         <b val="0"/>
@@ -4190,6 +4181,18 @@
     <dxf>
       <numFmt numFmtId="22" formatCode="mmm/yy"/>
     </dxf>
+    <dxf>
+      <numFmt numFmtId="175" formatCode="&quot;$&quot;#,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="175" formatCode="&quot;$&quot;#,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="175" formatCode="&quot;$&quot;#,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="22" formatCode="mmm/yy"/>
+    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
@@ -4213,11 +4216,11 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{0792567E-A03E-4943-98E4-EB876B9B20D6}" name="WaterfallData" displayName="WaterfallData" ref="A1:E8" totalsRowShown="0">
   <autoFilter ref="A1:E8" xr:uid="{0792567E-A03E-4943-98E4-EB876B9B20D6}"/>
   <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{E535E1E4-A65E-480E-B37A-792FC0723850}" name="Month" dataDxfId="3"/>
+    <tableColumn id="1" xr3:uid="{E535E1E4-A65E-480E-B37A-792FC0723850}" name="Month" dataDxfId="20"/>
     <tableColumn id="2" xr3:uid="{AF51F227-B625-4255-94A7-6199B7D7DAD1}" name="Movement"/>
-    <tableColumn id="3" xr3:uid="{72A4FA60-7150-4102-88DE-5B089CAE1D25}" name="Actual" dataDxfId="2"/>
-    <tableColumn id="4" xr3:uid="{69CC0EB6-9154-4E79-8DD0-FAB442AC9657}" name="Forecast" dataDxfId="1"/>
-    <tableColumn id="5" xr3:uid="{4D5B15AB-1D25-4871-B2A0-95F16E574BA9}" name="Variance" dataDxfId="0"/>
+    <tableColumn id="3" xr3:uid="{72A4FA60-7150-4102-88DE-5B089CAE1D25}" name="Actual" dataDxfId="19"/>
+    <tableColumn id="4" xr3:uid="{69CC0EB6-9154-4E79-8DD0-FAB442AC9657}" name="Forecast" dataDxfId="18"/>
+    <tableColumn id="5" xr3:uid="{4D5B15AB-1D25-4871-B2A0-95F16E574BA9}" name="Variance" dataDxfId="17"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -4232,8 +4235,8 @@
     <tableColumn id="3" xr3:uid="{3945ECD4-BB6F-4E5B-9B54-0517BF942829}" name="customer_id"/>
     <tableColumn id="4" xr3:uid="{82CA9B0A-4810-468C-8854-3017D97B8592}" name="company_name"/>
     <tableColumn id="5" xr3:uid="{30A8D838-4B8E-4217-8666-E0DF4BB06955}" name="region"/>
-    <tableColumn id="6" xr3:uid="{D841C5AC-D4B5-409A-8CFA-53443E346DCF}" name="month" dataDxfId="20"/>
-    <tableColumn id="7" xr3:uid="{6DBCDEDE-28AB-45B0-93DD-BA33B3BFB675}" name="event_date" dataDxfId="19"/>
+    <tableColumn id="6" xr3:uid="{D841C5AC-D4B5-409A-8CFA-53443E346DCF}" name="month" dataDxfId="16"/>
+    <tableColumn id="7" xr3:uid="{6DBCDEDE-28AB-45B0-93DD-BA33B3BFB675}" name="event_date" dataDxfId="15"/>
     <tableColumn id="8" xr3:uid="{C44CB2B9-5967-4692-A03A-7AF3E634A147}" name="event_type"/>
     <tableColumn id="9" xr3:uid="{47B2CD92-F52F-435B-8F19-D30BF4C73CE3}" name="old_value"/>
     <tableColumn id="10" xr3:uid="{5E6457F7-8D2B-4A6E-BB02-89A98B1FF9A9}" name="new_value"/>
@@ -4247,7 +4250,7 @@
     <tableColumn id="18" xr3:uid="{1FFE8D74-8F15-43CF-B8E5-E408F0044790}" name="movement">
       <calculatedColumnFormula array="1">_xlfn.IFS(H2="created", "New", H2="cancelled", "Churned", AND(H2="seats_change", J2 &gt; I2), "Expansion", AND(H2="seats_change", J2 &lt; I2), "Contraction", AND(H2="price_change", J2 &gt; I2), "Expansion", AND(H2="price_change", J2 &lt; I2), "Contraction", H2="plan_upgrade", "Expansion", H2="plan_downgrade", "Contraction", H2="discount_added", "Contraction")</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="19" xr3:uid="{543176F6-F2BB-4A01-87F5-5C68A679C2B3}" name="mrr_delta" dataDxfId="18">
+    <tableColumn id="19" xr3:uid="{543176F6-F2BB-4A01-87F5-5C68A679C2B3}" name="mrr_delta" dataDxfId="14">
       <calculatedColumnFormula array="1">IF(N2="Monthly",_xlfn.IFS(H2="created",O2*P2*(1-Q2/100),H2="cancelled",-(O2*P2*(1-Q2/100)),H2="seats_change",(J2-I2)*P2*(1-Q2/100),H2="price_change",(J2-I2)*O2*(1-Q2/100),H2="discount_added",-(O2*P2*(J2-I2)/100),H2="plan_upgrade",O2*(_xlfn.XLOOKUP(J2,$M:$M,$P:$P)-_xlfn.XLOOKUP(I2,$M:$M,$P:$P))*(1-Q2/100),H2="plan_downgrade",O2*(_xlfn.XLOOKUP(J2,$M:$M,$P:$P)-_xlfn.XLOOKUP(I2,$M:$M,$P:$P))*(1-Q2/100)),_xlfn.IFS(H2="created",O2*P2*(1-Q2/100)/12,H2="cancelled",-(O2*P2*(1-Q2/100))/12,H2="seats_change",(J2-I2)*P2*(1-Q2/100)/12,H2="price_change",(J2-I2)*O2*(1-Q2/100)/12,H2="plan_upgrade",(O2*(_xlfn.XLOOKUP(J2,$M:$M,$P:$P)-_xlfn.XLOOKUP(I2,$M:$M,$P:$P))*(1-Q2/100))/12,H2="plan_downgrade",(O2*(_xlfn.XLOOKUP(J2,$M:$M,$P:$P)-_xlfn.XLOOKUP(I2,$M:$M,$P:$P))*(1-Q2/100))/12,H2="discount_added",-(O2*P2*(J2-I2)/100)/12))</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -4256,19 +4259,19 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{539C435F-C1A6-4146-89EF-73537E96D5A1}" name="SMSpend" displayName="SMSpend" ref="A66:J80" totalsRowShown="0" headerRowDxfId="17" dataDxfId="16">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{539C435F-C1A6-4146-89EF-73537E96D5A1}" name="SMSpend" displayName="SMSpend" ref="A66:J80" totalsRowShown="0" headerRowDxfId="13" dataDxfId="12">
   <autoFilter ref="A66:J80" xr:uid="{B4D1F123-2972-489C-8FEC-9C6D26BDA440}"/>
   <tableColumns count="10">
-    <tableColumn id="1" xr3:uid="{428B9524-495F-4624-8292-AC7281BC37CF}" name="Month" dataDxfId="15"/>
-    <tableColumn id="2" xr3:uid="{A39BE488-44BB-4D32-8BC9-2CAD0287B7FB}" name="Sales Comp" dataDxfId="14"/>
-    <tableColumn id="3" xr3:uid="{5A5033F7-6D0F-4017-B24D-2EF30AF0C04A}" name="Marketing Comp" dataDxfId="13"/>
-    <tableColumn id="4" xr3:uid="{221D6297-6EAF-44F9-9192-FCE924DEAE38}" name="Paid Ads" dataDxfId="12"/>
-    <tableColumn id="5" xr3:uid="{DDDAF5EF-D699-4B54-AE9C-1DE1AE53E1FA}" name="Content &amp; SEO" dataDxfId="11"/>
-    <tableColumn id="6" xr3:uid="{C06DAFB6-3F41-4AB7-AC72-F2CD13738214}" name="Partner Commissions" dataDxfId="10"/>
-    <tableColumn id="7" xr3:uid="{B2373C96-3DA9-4205-B260-ECD2E8248D4F}" name="Tools &amp; Software" dataDxfId="9"/>
-    <tableColumn id="8" xr3:uid="{4C8B3A2D-C15B-426C-8B89-E7B5EA3AC7A8}" name="Events" dataDxfId="8"/>
-    <tableColumn id="9" xr3:uid="{591DAA16-7C9D-4A8A-8098-00ABCE2C68AB}" name="Total S&amp;M" dataDxfId="7"/>
-    <tableColumn id="10" xr3:uid="{27267743-1105-471C-A056-7EE8466EDA53}" name="New Customers" dataDxfId="6"/>
+    <tableColumn id="1" xr3:uid="{428B9524-495F-4624-8292-AC7281BC37CF}" name="Month" dataDxfId="11"/>
+    <tableColumn id="2" xr3:uid="{A39BE488-44BB-4D32-8BC9-2CAD0287B7FB}" name="Sales Comp" dataDxfId="10"/>
+    <tableColumn id="3" xr3:uid="{5A5033F7-6D0F-4017-B24D-2EF30AF0C04A}" name="Marketing Comp" dataDxfId="9"/>
+    <tableColumn id="4" xr3:uid="{221D6297-6EAF-44F9-9192-FCE924DEAE38}" name="Paid Ads" dataDxfId="8"/>
+    <tableColumn id="5" xr3:uid="{DDDAF5EF-D699-4B54-AE9C-1DE1AE53E1FA}" name="Content &amp; SEO" dataDxfId="7"/>
+    <tableColumn id="6" xr3:uid="{C06DAFB6-3F41-4AB7-AC72-F2CD13738214}" name="Partner Commissions" dataDxfId="6"/>
+    <tableColumn id="7" xr3:uid="{B2373C96-3DA9-4205-B260-ECD2E8248D4F}" name="Tools &amp; Software" dataDxfId="5"/>
+    <tableColumn id="8" xr3:uid="{4C8B3A2D-C15B-426C-8B89-E7B5EA3AC7A8}" name="Events" dataDxfId="4"/>
+    <tableColumn id="9" xr3:uid="{591DAA16-7C9D-4A8A-8098-00ABCE2C68AB}" name="Total S&amp;M" dataDxfId="3"/>
+    <tableColumn id="10" xr3:uid="{27267743-1105-471C-A056-7EE8466EDA53}" name="New Customers" dataDxfId="2"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -4280,8 +4283,8 @@
   <tableColumns count="4">
     <tableColumn id="1" xr3:uid="{01F66372-C956-4E27-89CF-1874F2147DCD}" name="plan_name"/>
     <tableColumn id="2" xr3:uid="{CCAD8762-EF12-4CFA-B5B5-C51B5EADA2B4}" name="monthly_price"/>
-    <tableColumn id="3" xr3:uid="{C40B4B1D-B122-4F11-B805-69D33B9BC9E8}" name="monthly_cost" dataDxfId="5"/>
-    <tableColumn id="4" xr3:uid="{9C412AFC-8F05-4E39-B8E1-9E65F1E3A073}" name="gross_margin" dataDxfId="4"/>
+    <tableColumn id="3" xr3:uid="{C40B4B1D-B122-4F11-B805-69D33B9BC9E8}" name="monthly_cost" dataDxfId="1"/>
+    <tableColumn id="4" xr3:uid="{9C412AFC-8F05-4E39-B8E1-9E65F1E3A073}" name="gross_margin" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -5835,30 +5838,30 @@
       <c r="A47" s="7" t="s">
         <v>70</v>
       </c>
-      <c r="B47" s="112" t="s">
+      <c r="B47" s="126" t="s">
         <v>311</v>
       </c>
-      <c r="C47" s="112"/>
-      <c r="D47" s="112"/>
-      <c r="E47" s="112"/>
-      <c r="F47" s="112"/>
-      <c r="G47" s="112"/>
-      <c r="H47" s="112"/>
-      <c r="I47" s="112"/>
+      <c r="C47" s="126"/>
+      <c r="D47" s="126"/>
+      <c r="E47" s="126"/>
+      <c r="F47" s="126"/>
+      <c r="G47" s="126"/>
+      <c r="H47" s="126"/>
+      <c r="I47" s="126"/>
     </row>
     <row r="49" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A49" s="15" t="s">
         <v>71</v>
       </c>
-      <c r="B49" s="112" t="s">
+      <c r="B49" s="126" t="s">
         <v>312</v>
       </c>
-      <c r="C49" s="112"/>
-      <c r="D49" s="112"/>
-      <c r="E49" s="112"/>
-      <c r="F49" s="112"/>
-      <c r="G49" s="112"/>
-      <c r="H49" s="112"/>
+      <c r="C49" s="126"/>
+      <c r="D49" s="126"/>
+      <c r="E49" s="126"/>
+      <c r="F49" s="126"/>
+      <c r="G49" s="126"/>
+      <c r="H49" s="126"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -6582,18 +6585,18 @@
       </c>
     </row>
     <row r="64" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A64" s="115" t="s">
+      <c r="A64" s="129" t="s">
         <v>256</v>
       </c>
-      <c r="B64" s="115"/>
-      <c r="C64" s="115"/>
-      <c r="D64" s="115"/>
-      <c r="E64" s="115"/>
-      <c r="F64" s="115"/>
-      <c r="G64" s="115"/>
-      <c r="H64" s="115"/>
-      <c r="I64" s="115"/>
-      <c r="J64" s="115"/>
+      <c r="B64" s="129"/>
+      <c r="C64" s="129"/>
+      <c r="D64" s="129"/>
+      <c r="E64" s="129"/>
+      <c r="F64" s="129"/>
+      <c r="G64" s="129"/>
+      <c r="H64" s="129"/>
+      <c r="I64" s="129"/>
+      <c r="J64" s="129"/>
     </row>
     <row r="65" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A65" s="62" t="s">
@@ -8625,7 +8628,7 @@
   <sheetPr>
     <tabColor rgb="FF7030A0"/>
   </sheetPr>
-  <dimension ref="A1:H65"/>
+  <dimension ref="A1:H66"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="32.7265625" customWidth="1"/>
@@ -8677,7 +8680,7 @@
         <v>0</v>
       </c>
       <c r="E3" s="101">
-        <f>B3/C3-1</f>
+        <f>IFERROR(B3/C3-1, 0)</f>
         <v>0</v>
       </c>
       <c r="F3" s="109" t="str" cm="1">
@@ -8696,11 +8699,11 @@
         <v>4000</v>
       </c>
       <c r="D4" s="25">
-        <f t="shared" ref="D4:D9" si="0">B4-C4</f>
+        <f t="shared" ref="D4:D10" si="0">B4-C4</f>
         <v>-2290</v>
       </c>
       <c r="E4" s="101">
-        <f t="shared" ref="E4:E6" si="1">B4/C4-1</f>
+        <f t="shared" ref="E4:E7" si="1">IFERROR(B4/C4-1, 0)</f>
         <v>-0.57250000000000001</v>
       </c>
       <c r="F4" s="109" t="str" cm="1">
@@ -8734,72 +8737,70 @@
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A6" s="7" t="s">
+        <v>655</v>
+      </c>
+      <c r="B6" s="25">
+        <v>0</v>
+      </c>
+      <c r="C6" s="25">
+        <v>0</v>
+      </c>
+      <c r="D6" s="25">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="E6" s="101">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="F6" s="109" t="str" cm="1">
+        <f t="array" ref="F6">_xlfn.IFS(D6&lt;0, "U", D6&gt;0, "F", D6=0, "-")</f>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A7" s="7" t="s">
         <v>22</v>
       </c>
-      <c r="B6" s="25">
-        <v>0</v>
-      </c>
-      <c r="C6" s="25">
+      <c r="B7" s="25">
+        <v>0</v>
+      </c>
+      <c r="C7" s="25">
         <f>'2026 Forecast'!B10/3</f>
         <v>953.79666666666662</v>
       </c>
-      <c r="D6" s="25">
+      <c r="D7" s="25">
         <f t="shared" si="0"/>
         <v>-953.79666666666662</v>
       </c>
-      <c r="E6" s="101">
+      <c r="E7" s="101">
         <f t="shared" si="1"/>
         <v>-1</v>
       </c>
-      <c r="F6" s="109" t="str" cm="1">
-        <f t="array" ref="F6">_xlfn.IFS(D6&gt;0, "U", D6&lt;0, "F", D6=0, "-")</f>
+      <c r="F7" s="109" t="str" cm="1">
+        <f t="array" ref="F7">_xlfn.IFS(D7&gt;0, "U", D7&lt;0, "F", D7=0, "-")</f>
         <v>F</v>
       </c>
     </row>
-    <row r="7" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A7" s="9" t="s">
+    <row r="8" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A8" s="9" t="s">
         <v>24</v>
       </c>
-      <c r="B7" s="26">
-        <f>B4+B5-B6</f>
+      <c r="B8" s="26">
+        <f>B4+B5-B7</f>
         <v>1710</v>
       </c>
-      <c r="C7" s="26">
-        <f>C4+C5-C6</f>
+      <c r="C8" s="26">
+        <f>C4+C5-C7</f>
         <v>3761.5508333333332</v>
       </c>
-      <c r="D7" s="26">
+      <c r="D8" s="26">
         <f t="shared" si="0"/>
         <v>-2051.5508333333332</v>
       </c>
-      <c r="E7" s="102">
-        <f>B7/C7-1</f>
-        <v>-0.54540026819611853</v>
-      </c>
-      <c r="F7" s="110" t="str" cm="1">
-        <f t="array" ref="F7">_xlfn.IFS(D7&lt;0, "U", D7&gt;0, "F", D7=0, "-")</f>
-        <v>U</v>
-      </c>
-    </row>
-    <row r="8" spans="1:8" ht="15.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A8" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="B8" s="26">
-        <f>B3+B4+B5-B6</f>
-        <v>144779.5</v>
-      </c>
-      <c r="C8" s="26">
-        <f>C3+C7</f>
-        <v>146831.05083333334</v>
-      </c>
-      <c r="D8" s="26">
-        <f t="shared" si="0"/>
-        <v>-2051.5508333333419</v>
-      </c>
       <c r="E8" s="102">
         <f>B8/C8-1</f>
-        <v>-1.3972186548348309E-2</v>
+        <v>-0.54540026819611853</v>
       </c>
       <c r="F8" s="110" t="str" cm="1">
         <f t="array" ref="F8">_xlfn.IFS(D8&lt;0, "U", D8&gt;0, "F", D8=0, "-")</f>
@@ -8808,19 +8809,19 @@
     </row>
     <row r="9" spans="1:8" ht="15.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A9" s="9" t="s">
-        <v>112</v>
+        <v>26</v>
       </c>
       <c r="B9" s="26">
-        <f>B8*12</f>
-        <v>1737354</v>
-      </c>
-      <c r="C9" s="22">
-        <f>C8*12</f>
-        <v>1761972.61</v>
-      </c>
-      <c r="D9" s="22">
+        <f>B3+B4+B5-B7</f>
+        <v>144779.5</v>
+      </c>
+      <c r="C9" s="26">
+        <f>C3+C8</f>
+        <v>146831.05083333334</v>
+      </c>
+      <c r="D9" s="26">
         <f t="shared" si="0"/>
-        <v>-24618.610000000102</v>
+        <v>-2051.5508333333419</v>
       </c>
       <c r="E9" s="102">
         <f>B9/C9-1</f>
@@ -8831,154 +8832,151 @@
         <v>U</v>
       </c>
     </row>
-    <row r="10" spans="1:8" ht="15" thickTop="1" x14ac:dyDescent="0.35"/>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A11" s="104" t="s">
+    <row r="10" spans="1:8" ht="15.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A10" s="9" t="s">
+        <v>112</v>
+      </c>
+      <c r="B10" s="26">
+        <f>B9*12</f>
+        <v>1737354</v>
+      </c>
+      <c r="C10" s="22">
+        <f>C9*12</f>
+        <v>1761972.61</v>
+      </c>
+      <c r="D10" s="22">
+        <f t="shared" si="0"/>
+        <v>-24618.610000000102</v>
+      </c>
+      <c r="E10" s="102">
+        <f>B10/C10-1</f>
+        <v>-1.3972186548348309E-2</v>
+      </c>
+      <c r="F10" s="110" t="str" cm="1">
+        <f t="array" ref="F10">_xlfn.IFS(D10&lt;0, "U", D10&gt;0, "F", D10=0, "-")</f>
+        <v>U</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" ht="15" thickTop="1" x14ac:dyDescent="0.35"/>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A12" s="104" t="s">
         <v>601</v>
       </c>
     </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A12" s="5" t="s">
+    <row r="13" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A13" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="B12" s="5" t="s">
+      <c r="B13" s="5" t="s">
         <v>599</v>
       </c>
-      <c r="C12" s="99" t="s">
+      <c r="C13" s="99" t="s">
         <v>596</v>
       </c>
-      <c r="D12" s="99" t="s">
+      <c r="D13" s="99" t="s">
         <v>597</v>
       </c>
-      <c r="E12" s="99" t="s">
+      <c r="E13" s="99" t="s">
         <v>598</v>
       </c>
-      <c r="F12" s="103" t="s">
+      <c r="F13" s="103" t="s">
         <v>602</v>
       </c>
-    </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A13" s="7" t="s">
-        <v>38</v>
-      </c>
-      <c r="B13" s="100">
-        <f>B8</f>
-        <v>144779.5</v>
-      </c>
-      <c r="C13" s="100">
-        <f>C8</f>
-        <v>146831.05083333334</v>
-      </c>
-      <c r="D13" s="100">
-        <f>B13-C13</f>
-        <v>-2051.5508333333419</v>
-      </c>
-      <c r="E13" s="105">
-        <f>B13/C13-1</f>
-        <v>-1.3972186548348309E-2</v>
-      </c>
-      <c r="F13" s="109" t="str" cm="1">
-        <f t="array" ref="F13">_xlfn.IFS(D13&lt;0, "U", D13&gt;0, "F", D13=0, "-")</f>
-        <v>U</v>
-      </c>
-      <c r="H13" s="2"/>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A14" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="B14" s="100">
+        <f>B9</f>
+        <v>144779.5</v>
+      </c>
+      <c r="C14" s="100">
+        <f>C9</f>
+        <v>146831.05083333334</v>
+      </c>
+      <c r="D14" s="100">
+        <f>B14-C14</f>
+        <v>-2051.5508333333419</v>
+      </c>
+      <c r="E14" s="105">
+        <f>B14/C14-1</f>
+        <v>-1.3972186548348309E-2</v>
+      </c>
+      <c r="F14" s="109" t="str" cm="1">
+        <f t="array" ref="F14">_xlfn.IFS(D14&lt;0, "U", D14&gt;0, "F", D14=0, "-")</f>
+        <v>U</v>
+      </c>
+      <c r="H14" s="2"/>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A15" s="7" t="s">
         <v>119</v>
       </c>
-      <c r="B14" s="100">
-        <f>B13*(1-B16)</f>
+      <c r="B15" s="100">
+        <f>B14*(1-B17)</f>
         <v>43433.850000000006</v>
       </c>
-      <c r="C14" s="100">
-        <f>C13*0.3</f>
+      <c r="C15" s="100">
+        <f>C14*0.3</f>
         <v>44049.31525</v>
       </c>
-      <c r="D14" s="100">
-        <f t="shared" ref="D14:D21" si="2">B14-C14</f>
+      <c r="D15" s="100">
+        <f t="shared" ref="D15:D22" si="2">B15-C15</f>
         <v>-615.46524999999383</v>
       </c>
-      <c r="E14" s="105">
-        <f t="shared" ref="E14:E22" si="3">B14/C14-1</f>
+      <c r="E15" s="105">
+        <f t="shared" ref="E15:E23" si="3">B15/C15-1</f>
         <v>-1.3972186548348087E-2</v>
       </c>
-      <c r="F14" s="109" t="str" cm="1">
-        <f t="array" ref="F14">_xlfn.IFS(D14&gt;0, "U", D14&lt;0, "F", D14=0, "-")</f>
+      <c r="F15" s="109" t="str" cm="1">
+        <f t="array" ref="F15">_xlfn.IFS(D15&gt;0, "U", D15&lt;0, "F", D15=0, "-")</f>
         <v>F</v>
       </c>
-      <c r="H14" s="2" t="s">
+      <c r="H15" s="2" t="s">
         <v>120</v>
       </c>
     </row>
-    <row r="15" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A15" s="9" t="s">
+    <row r="16" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A16" s="9" t="s">
         <v>42</v>
       </c>
-      <c r="B15" s="106">
-        <f>B13-B14</f>
+      <c r="B16" s="106">
+        <f>B14-B15</f>
         <v>101345.65</v>
       </c>
-      <c r="C15" s="106">
-        <f>C13-C14</f>
+      <c r="C16" s="106">
+        <f>C14-C15</f>
         <v>102781.73558333334</v>
       </c>
-      <c r="D15" s="100">
+      <c r="D16" s="100">
         <f t="shared" si="2"/>
         <v>-1436.085583333348</v>
       </c>
-      <c r="E15" s="105">
+      <c r="E16" s="105">
         <f t="shared" si="3"/>
         <v>-1.3972186548348309E-2</v>
       </c>
-      <c r="F15" s="109" t="str" cm="1">
-        <f t="array" ref="F15">_xlfn.IFS(D15&lt;0, "U", D15&gt;0, "F", D15=0, "-")</f>
-        <v>U</v>
-      </c>
-      <c r="H15" s="2" t="s">
-        <v>121</v>
-      </c>
-    </row>
-    <row r="16" spans="1:8" ht="15" thickTop="1" x14ac:dyDescent="0.35">
-      <c r="A16" s="7" t="s">
-        <v>44</v>
-      </c>
-      <c r="B16" s="108">
-        <v>0.7</v>
-      </c>
-      <c r="C16" s="105">
-        <f>C15/C13</f>
-        <v>0.70000000000000007</v>
-      </c>
-      <c r="D16" s="100"/>
-      <c r="E16" s="105">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
       <c r="F16" s="109" t="str" cm="1">
         <f t="array" ref="F16">_xlfn.IFS(D16&lt;0, "U", D16&gt;0, "F", D16=0, "-")</f>
-        <v>-</v>
+        <v>U</v>
       </c>
       <c r="H16" s="2" t="s">
-        <v>122</v>
-      </c>
-    </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.35">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8" ht="15" thickTop="1" x14ac:dyDescent="0.35">
       <c r="A17" s="7" t="s">
-        <v>94</v>
-      </c>
-      <c r="B17" s="100">
-        <f>'Forecast Assumptions'!B26/3</f>
-        <v>30000</v>
-      </c>
-      <c r="C17" s="100">
-        <f>'2026 Forecast'!B25/3</f>
-        <v>30000</v>
-      </c>
-      <c r="D17" s="100">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
+        <v>44</v>
+      </c>
+      <c r="B17" s="108">
+        <v>0.7</v>
+      </c>
+      <c r="C17" s="105">
+        <f>C16/C14</f>
+        <v>0.70000000000000007</v>
+      </c>
+      <c r="D17" s="100"/>
       <c r="E17" s="105">
         <f t="shared" si="3"/>
         <v>0</v>
@@ -8988,20 +8986,20 @@
         <v>-</v>
       </c>
       <c r="H17" s="2" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
     </row>
     <row r="18" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A18" s="7" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="B18" s="100">
-        <f>'Forecast Assumptions'!B27/3</f>
-        <v>25000</v>
+        <f>'Forecast Assumptions'!B26/3</f>
+        <v>30000</v>
       </c>
       <c r="C18" s="100">
-        <f>'2026 Forecast'!B26/3</f>
-        <v>25000</v>
+        <f>'2026 Forecast'!B25/3</f>
+        <v>30000</v>
       </c>
       <c r="D18" s="100">
         <f t="shared" si="2"/>
@@ -9021,15 +9019,15 @@
     </row>
     <row r="19" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A19" s="7" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="B19" s="100">
-        <f>'Forecast Assumptions'!B28/3</f>
-        <v>19000</v>
+        <f>'Forecast Assumptions'!B27/3</f>
+        <v>25000</v>
       </c>
       <c r="C19" s="100">
-        <f>'2026 Forecast'!B27/3</f>
-        <v>19000</v>
+        <f>'2026 Forecast'!B26/3</f>
+        <v>25000</v>
       </c>
       <c r="D19" s="100">
         <f t="shared" si="2"/>
@@ -9047,17 +9045,17 @@
         <v>123</v>
       </c>
     </row>
-    <row r="20" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A20" s="9" t="s">
-        <v>51</v>
-      </c>
-      <c r="B20" s="106">
-        <f>SUM(B17:B19)</f>
-        <v>74000</v>
-      </c>
-      <c r="C20" s="106">
-        <f>'2026 Forecast'!B28/3</f>
-        <v>74000</v>
+    <row r="20" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A20" s="7" t="s">
+        <v>96</v>
+      </c>
+      <c r="B20" s="100">
+        <f>'Forecast Assumptions'!B28/3</f>
+        <v>19000</v>
+      </c>
+      <c r="C20" s="100">
+        <f>'2026 Forecast'!B27/3</f>
+        <v>19000</v>
       </c>
       <c r="D20" s="100">
         <f t="shared" si="2"/>
@@ -9072,148 +9070,165 @@
         <v>-</v>
       </c>
       <c r="H20" s="2" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="21" spans="1:8" ht="15.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="21" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A21" s="9" t="s">
-        <v>53</v>
-      </c>
-      <c r="B21" s="107">
-        <f>B15-B20</f>
-        <v>27345.649999999994</v>
-      </c>
-      <c r="C21" s="107">
-        <f>C15-C20</f>
-        <v>28781.735583333342</v>
+        <v>51</v>
+      </c>
+      <c r="B21" s="106">
+        <f>SUM(B18:B20)</f>
+        <v>74000</v>
+      </c>
+      <c r="C21" s="106">
+        <f>'2026 Forecast'!B28/3</f>
+        <v>74000</v>
       </c>
       <c r="D21" s="100">
         <f t="shared" si="2"/>
-        <v>-1436.085583333348</v>
+        <v>0</v>
       </c>
       <c r="E21" s="105">
         <f t="shared" si="3"/>
-        <v>-4.9895725682538195E-2</v>
+        <v>0</v>
       </c>
       <c r="F21" s="109" t="str" cm="1">
         <f t="array" ref="F21">_xlfn.IFS(D21&lt;0, "U", D21&gt;0, "F", D21=0, "-")</f>
-        <v>U</v>
+        <v>-</v>
       </c>
       <c r="H21" s="2" t="s">
-        <v>124</v>
-      </c>
-    </row>
-    <row r="22" spans="1:8" ht="15" thickTop="1" x14ac:dyDescent="0.35">
-      <c r="A22" s="7" t="s">
-        <v>55</v>
-      </c>
-      <c r="B22" s="105">
-        <f>B21/B13</f>
-        <v>0.18887791434560827</v>
-      </c>
-      <c r="C22" s="105">
-        <f>C21/C13</f>
-        <v>0.19601940747535235</v>
-      </c>
-      <c r="D22" s="105">
-        <f>B22-C22</f>
-        <v>-7.1414931297440754E-3</v>
+        <v>52</v>
+      </c>
+    </row>
+    <row r="22" spans="1:8" ht="15.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A22" s="9" t="s">
+        <v>53</v>
+      </c>
+      <c r="B22" s="107">
+        <f>B16-B21</f>
+        <v>27345.649999999994</v>
+      </c>
+      <c r="C22" s="107">
+        <f>C16-C21</f>
+        <v>28781.735583333342</v>
+      </c>
+      <c r="D22" s="100">
+        <f t="shared" si="2"/>
+        <v>-1436.085583333348</v>
       </c>
       <c r="E22" s="105">
         <f t="shared" si="3"/>
-        <v>-3.643258196585486E-2</v>
+        <v>-4.9895725682538195E-2</v>
       </c>
       <c r="F22" s="109" t="str" cm="1">
         <f t="array" ref="F22">_xlfn.IFS(D22&lt;0, "U", D22&gt;0, "F", D22=0, "-")</f>
         <v>U</v>
       </c>
       <c r="H22" s="2" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="23" spans="1:8" ht="15" thickTop="1" x14ac:dyDescent="0.35">
+      <c r="A23" s="7" t="s">
+        <v>55</v>
+      </c>
+      <c r="B23" s="105">
+        <f>B22/B14</f>
+        <v>0.18887791434560827</v>
+      </c>
+      <c r="C23" s="105">
+        <f>C22/C14</f>
+        <v>0.19601940747535235</v>
+      </c>
+      <c r="D23" s="105">
+        <f>B23-C23</f>
+        <v>-7.1414931297440754E-3</v>
+      </c>
+      <c r="E23" s="105">
+        <f t="shared" si="3"/>
+        <v>-3.643258196585486E-2</v>
+      </c>
+      <c r="F23" s="109" t="str" cm="1">
+        <f t="array" ref="F23">_xlfn.IFS(D23&lt;0, "U", D23&gt;0, "F", D23=0, "-")</f>
+        <v>U</v>
+      </c>
+      <c r="H23" s="2" t="s">
         <v>125</v>
       </c>
     </row>
-    <row r="24" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A24" s="111" t="s">
+    <row r="25" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A25" s="111" t="s">
         <v>611</v>
-      </c>
-    </row>
-    <row r="25" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A25" t="s">
-        <v>603</v>
       </c>
     </row>
     <row r="26" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
-        <v>604</v>
+        <v>603</v>
       </c>
     </row>
     <row r="27" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
-        <v>605</v>
+        <v>604</v>
       </c>
     </row>
     <row r="28" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
-        <v>612</v>
+        <v>605</v>
       </c>
     </row>
     <row r="29" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
-        <v>607</v>
+        <v>612</v>
       </c>
     </row>
     <row r="30" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
-        <v>606</v>
+        <v>607</v>
       </c>
     </row>
     <row r="31" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
-        <v>609</v>
+        <v>606</v>
       </c>
     </row>
     <row r="32" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
-        <v>608</v>
+        <v>609</v>
       </c>
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
+        <v>608</v>
+      </c>
+    </row>
+    <row r="34" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A34" t="s">
         <v>610</v>
       </c>
     </row>
-    <row r="35" spans="1:3" ht="17" x14ac:dyDescent="0.4">
-      <c r="A35" s="116" t="s">
+    <row r="36" spans="1:3" ht="17" x14ac:dyDescent="0.4">
+      <c r="A36" s="112" t="s">
         <v>613</v>
       </c>
     </row>
-    <row r="37" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A37" s="117" t="s">
+    <row r="38" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A38" s="113" t="s">
         <v>4</v>
       </c>
-      <c r="B37" s="117" t="s">
+      <c r="B38" s="113" t="s">
         <v>283</v>
       </c>
-      <c r="C37" s="117" t="s">
+      <c r="C38" s="113" t="s">
         <v>614</v>
-      </c>
-    </row>
-    <row r="38" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A38" t="s">
-        <v>193</v>
-      </c>
-      <c r="B38" s="118">
-        <v>39</v>
-      </c>
-      <c r="C38" t="s">
-        <v>615</v>
       </c>
     </row>
     <row r="39" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A39" t="s">
-        <v>194</v>
-      </c>
-      <c r="B39" s="118">
-        <v>52</v>
+        <v>193</v>
+      </c>
+      <c r="B39" s="114">
+        <v>39</v>
       </c>
       <c r="C39" t="s">
         <v>615</v>
@@ -9221,101 +9236,101 @@
     </row>
     <row r="40" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A40" t="s">
-        <v>616</v>
-      </c>
-      <c r="B40" s="100">
-        <f>'Unit Economics'!B7</f>
-        <v>3604.6374999999998</v>
+        <v>194</v>
+      </c>
+      <c r="B40" s="114">
+        <v>52</v>
       </c>
       <c r="C40" t="s">
-        <v>617</v>
+        <v>615</v>
       </c>
     </row>
     <row r="41" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A41" t="s">
-        <v>618</v>
-      </c>
-      <c r="B41" s="28">
-        <f>B16</f>
-        <v>0.7</v>
+        <v>616</v>
+      </c>
+      <c r="B41" s="100">
+        <f>'Jan 2026 A vs F '!B9/'Jan 2026 A vs F '!B39</f>
+        <v>3712.2948717948716</v>
       </c>
       <c r="C41" t="s">
-        <v>619</v>
+        <v>617</v>
       </c>
     </row>
     <row r="42" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A42" t="s">
+        <v>618</v>
+      </c>
+      <c r="B42" s="28">
+        <f>B17</f>
+        <v>0.7</v>
+      </c>
+      <c r="C42" t="s">
+        <v>619</v>
+      </c>
+    </row>
+    <row r="43" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A43" t="s">
         <v>620</v>
       </c>
-      <c r="B42" s="28">
+      <c r="B43" s="28">
         <f>Retention!Z6</f>
         <v>1</v>
       </c>
-      <c r="C42" t="s">
+      <c r="C43" t="s">
         <v>621</v>
       </c>
     </row>
-    <row r="43" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A43" t="s">
+    <row r="44" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A44" t="s">
         <v>622</v>
       </c>
-      <c r="B43" s="28">
+      <c r="B44" s="28">
         <f>Retention!Z7</f>
         <v>1</v>
       </c>
-      <c r="C43" t="s">
+      <c r="C44" t="s">
         <v>621</v>
-      </c>
-    </row>
-    <row r="44" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A44" t="s">
-        <v>623</v>
-      </c>
-      <c r="B44" t="s">
-        <v>624</v>
-      </c>
-      <c r="C44" t="s">
-        <v>654</v>
       </c>
     </row>
     <row r="45" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A45" t="s">
-        <v>625</v>
-      </c>
-      <c r="B45" s="44">
-        <f>B17</f>
-        <v>30000</v>
+        <v>623</v>
+      </c>
+      <c r="B45" t="s">
+        <v>624</v>
       </c>
       <c r="C45" t="s">
-        <v>626</v>
+        <v>654</v>
       </c>
     </row>
     <row r="46" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A46" t="s">
-        <v>627</v>
+        <v>625</v>
       </c>
       <c r="B46" s="44">
-        <f>B45/1</f>
+        <f>B18</f>
         <v>30000</v>
       </c>
       <c r="C46" t="s">
-        <v>637</v>
+        <v>626</v>
       </c>
     </row>
     <row r="47" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A47" t="s">
-        <v>628</v>
-      </c>
-      <c r="B47" t="s">
-        <v>629</v>
+        <v>627</v>
+      </c>
+      <c r="B47" s="44">
+        <f>B46/1</f>
+        <v>30000</v>
       </c>
       <c r="C47" t="s">
-        <v>630</v>
+        <v>637</v>
       </c>
     </row>
     <row r="48" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A48" t="s">
-        <v>631</v>
+        <v>628</v>
       </c>
       <c r="B48" t="s">
         <v>629</v>
@@ -9326,7 +9341,7 @@
     </row>
     <row r="49" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A49" t="s">
-        <v>632</v>
+        <v>631</v>
       </c>
       <c r="B49" t="s">
         <v>629</v>
@@ -9335,60 +9350,62 @@
         <v>630</v>
       </c>
     </row>
-    <row r="51" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A51" s="119" t="s">
+    <row r="50" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A50" t="s">
+        <v>632</v>
+      </c>
+      <c r="B50" t="s">
+        <v>629</v>
+      </c>
+      <c r="C50" t="s">
+        <v>630</v>
+      </c>
+    </row>
+    <row r="52" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A52" s="115" t="s">
         <v>633</v>
       </c>
     </row>
-    <row r="52" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A52" s="119" t="s">
+    <row r="53" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A53" s="115" t="s">
         <v>634</v>
       </c>
     </row>
-    <row r="54" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A54" s="119" t="s">
+    <row r="55" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A55" s="115" t="s">
         <v>635</v>
       </c>
     </row>
-    <row r="55" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A55" s="119" t="s">
+    <row r="56" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A56" s="115" t="s">
         <v>636</v>
       </c>
     </row>
-    <row r="58" spans="1:3" ht="17" x14ac:dyDescent="0.4">
-      <c r="A58" s="120" t="s">
+    <row r="59" spans="1:3" ht="17" x14ac:dyDescent="0.4">
+      <c r="A59" s="116" t="s">
         <v>638</v>
       </c>
     </row>
-    <row r="60" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A60" s="117" t="s">
+    <row r="61" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A61" s="113" t="s">
         <v>4</v>
       </c>
-      <c r="B60" s="117" t="s">
+      <c r="B61" s="113" t="s">
         <v>639</v>
-      </c>
-    </row>
-    <row r="61" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A61" t="s">
-        <v>616</v>
-      </c>
-      <c r="B61" s="100">
-        <f>B40</f>
-        <v>3604.6374999999998</v>
       </c>
     </row>
     <row r="62" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A62" t="s">
-        <v>620</v>
-      </c>
-      <c r="B62" s="28">
-        <f>B42</f>
-        <v>1</v>
+        <v>616</v>
+      </c>
+      <c r="B62" s="100">
+        <f>B41</f>
+        <v>3712.2948717948716</v>
       </c>
     </row>
     <row r="63" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A63" t="s">
-        <v>622</v>
+        <v>620</v>
       </c>
       <c r="B63" s="28">
         <f>B43</f>
@@ -9397,19 +9414,28 @@
     </row>
     <row r="64" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A64" t="s">
-        <v>623</v>
-      </c>
-      <c r="B64" t="str">
+        <v>622</v>
+      </c>
+      <c r="B64" s="28">
         <f>B44</f>
-        <v>N/A — no losses</v>
+        <v>1</v>
       </c>
     </row>
     <row r="65" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A65" t="s">
+        <v>623</v>
+      </c>
+      <c r="B65" t="str">
+        <f>B45</f>
+        <v>N/A — no losses</v>
+      </c>
+    </row>
+    <row r="66" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A66" t="s">
         <v>640</v>
       </c>
-      <c r="B65" s="44">
-        <f>B46</f>
+      <c r="B66" s="44">
+        <f>B47</f>
         <v>30000</v>
       </c>
     </row>
@@ -9417,7 +9443,7 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
   <ignoredErrors>
-    <ignoredError sqref="F6 F14" formula="1"/>
+    <ignoredError sqref="F7 F15" formula="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -9436,24 +9462,24 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="18.5" x14ac:dyDescent="0.45">
-      <c r="A1" s="121" t="s">
+      <c r="A1" s="117" t="s">
         <v>641</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A3" s="117" t="s">
+      <c r="A3" s="113" t="s">
         <v>4</v>
       </c>
-      <c r="B3" s="122">
+      <c r="B3" s="118">
         <v>46023</v>
       </c>
-      <c r="C3" s="122">
+      <c r="C3" s="118">
         <v>46054</v>
       </c>
-      <c r="D3" s="122">
+      <c r="D3" s="118">
         <v>46082</v>
       </c>
-      <c r="E3" s="123" t="s">
+      <c r="E3" s="119" t="s">
         <v>81</v>
       </c>
     </row>
@@ -9462,167 +9488,167 @@
         <v>26</v>
       </c>
       <c r="B4" s="100">
-        <f>'Jan 2026 A vs F '!B8</f>
+        <f>'Jan 2026 A vs F '!B9</f>
         <v>144779.5</v>
       </c>
-      <c r="E4" s="124"/>
+      <c r="E4" s="120"/>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>193</v>
       </c>
-      <c r="B5" s="125">
-        <f>'Jan 2026 A vs F '!B38</f>
+      <c r="B5" s="121">
+        <f>'Jan 2026 A vs F '!B39</f>
         <v>39</v>
       </c>
-      <c r="E5" s="124"/>
+      <c r="E5" s="120"/>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>616</v>
       </c>
       <c r="B6" s="100">
-        <f>'Jan 2026 A vs F '!B40</f>
-        <v>3604.6374999999998</v>
-      </c>
-      <c r="E6" s="124"/>
+        <f>'Jan 2026 A vs F '!B41</f>
+        <v>3712.2948717948716</v>
+      </c>
+      <c r="E6" s="120"/>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>618</v>
       </c>
       <c r="B7" s="28">
-        <f>'Jan 2026 A vs F '!B41</f>
+        <f>'Jan 2026 A vs F '!B42</f>
         <v>0.7</v>
       </c>
-      <c r="E7" s="124"/>
+      <c r="E7" s="120"/>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>620</v>
       </c>
       <c r="B8" s="28">
-        <f>'Jan 2026 A vs F '!B42</f>
+        <f>'Jan 2026 A vs F '!B43</f>
         <v>1</v>
       </c>
-      <c r="E8" s="124"/>
+      <c r="E8" s="120"/>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>622</v>
       </c>
       <c r="B9" s="28">
-        <f>'Jan 2026 A vs F '!B43</f>
+        <f>'Jan 2026 A vs F '!B44</f>
         <v>1</v>
       </c>
-      <c r="E9" s="124"/>
+      <c r="E9" s="120"/>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>623</v>
       </c>
       <c r="B10" t="str">
-        <f>'Jan 2026 A vs F '!B44</f>
+        <f>'Jan 2026 A vs F '!B45</f>
         <v>N/A — no losses</v>
       </c>
-      <c r="E10" s="124"/>
+      <c r="E10" s="120"/>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>625</v>
       </c>
       <c r="B11" s="44">
-        <f>'Jan 2026 A vs F '!B45</f>
+        <f>'Jan 2026 A vs F '!B46</f>
         <v>30000</v>
       </c>
-      <c r="E11" s="124"/>
+      <c r="E11" s="120"/>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>642</v>
       </c>
       <c r="B12" s="44">
-        <f>'Jan 2026 A vs F '!B46</f>
+        <f>'Jan 2026 A vs F '!B47</f>
         <v>30000</v>
       </c>
-      <c r="E12" s="124"/>
+      <c r="E12" s="120"/>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A13" s="124" t="s">
+      <c r="A13" s="120" t="s">
         <v>643</v>
       </c>
-      <c r="B13" s="126" t="s">
+      <c r="B13" s="122" t="s">
         <v>629</v>
       </c>
-      <c r="C13" s="126" t="s">
+      <c r="C13" s="122" t="s">
         <v>629</v>
       </c>
-      <c r="D13" s="126" t="s">
+      <c r="D13" s="122" t="s">
         <v>629</v>
       </c>
-      <c r="E13" s="127" t="s">
+      <c r="E13" s="123" t="s">
         <v>644</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A14" s="124" t="s">
+      <c r="A14" s="120" t="s">
         <v>628</v>
       </c>
-      <c r="B14" s="126" t="s">
+      <c r="B14" s="122" t="s">
         <v>629</v>
       </c>
-      <c r="C14" s="126" t="s">
+      <c r="C14" s="122" t="s">
         <v>629</v>
       </c>
-      <c r="D14" s="126" t="s">
+      <c r="D14" s="122" t="s">
         <v>629</v>
       </c>
-      <c r="E14" s="127" t="s">
+      <c r="E14" s="123" t="s">
         <v>644</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A15" s="124" t="s">
+      <c r="A15" s="120" t="s">
         <v>631</v>
       </c>
-      <c r="B15" s="126" t="s">
+      <c r="B15" s="122" t="s">
         <v>629</v>
       </c>
-      <c r="C15" s="126" t="s">
+      <c r="C15" s="122" t="s">
         <v>629</v>
       </c>
-      <c r="D15" s="126" t="s">
+      <c r="D15" s="122" t="s">
         <v>629</v>
       </c>
-      <c r="E15" s="127" t="s">
+      <c r="E15" s="123" t="s">
         <v>644</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A16" s="124" t="s">
+      <c r="A16" s="120" t="s">
         <v>632</v>
       </c>
-      <c r="B16" s="126" t="s">
+      <c r="B16" s="122" t="s">
         <v>629</v>
       </c>
-      <c r="C16" s="126" t="s">
+      <c r="C16" s="122" t="s">
         <v>629</v>
       </c>
-      <c r="D16" s="126" t="s">
+      <c r="D16" s="122" t="s">
         <v>629</v>
       </c>
-      <c r="E16" s="127" t="s">
+      <c r="E16" s="123" t="s">
         <v>644</v>
       </c>
     </row>
     <row r="18" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A18" s="129" t="s">
+      <c r="A18" s="125" t="s">
         <v>645</v>
       </c>
-      <c r="B18" s="129"/>
-      <c r="C18" s="129"/>
-      <c r="D18" s="128"/>
-      <c r="E18" s="128"/>
+      <c r="B18" s="125"/>
+      <c r="C18" s="125"/>
+      <c r="D18" s="124"/>
+      <c r="E18" s="124"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -9731,10 +9757,11 @@
         <v>652</v>
       </c>
       <c r="C5" s="100">
-        <f>Waterfall!E27</f>
+        <f>'Jan 2026 A vs F '!B6</f>
         <v>0</v>
       </c>
       <c r="D5" s="100">
+        <f>'Jan 2026 A vs F '!C6</f>
         <v>0</v>
       </c>
       <c r="E5" s="100">
@@ -9750,11 +9777,11 @@
         <v>653</v>
       </c>
       <c r="C6" s="100">
-        <f>Waterfall!F27</f>
+        <f>'Jan 2026 A vs F '!B7</f>
         <v>0</v>
       </c>
       <c r="D6" s="100">
-        <f>'Jan 2026 A vs F '!C6</f>
+        <f>'Jan 2026 A vs F '!C7</f>
         <v>953.79666666666662</v>
       </c>
       <c r="E6" s="100">
@@ -9770,15 +9797,15 @@
         <v>24</v>
       </c>
       <c r="C7" s="100">
-        <f>'Jan 2026 A vs F '!B7</f>
+        <f>'Jan 2026 A vs F '!B8</f>
         <v>1710</v>
       </c>
       <c r="D7" s="100">
-        <f>'Jan 2026 A vs F '!C7</f>
+        <f>'Jan 2026 A vs F '!C8</f>
         <v>3761.5508333333332</v>
       </c>
       <c r="E7" s="100">
-        <f>'Jan 2026 A vs F '!D7</f>
+        <f>'Jan 2026 A vs F '!D8</f>
         <v>-2051.5508333333332</v>
       </c>
     </row>
@@ -9790,15 +9817,15 @@
         <v>26</v>
       </c>
       <c r="C8" s="100">
-        <f>'Jan 2026 A vs F '!B8</f>
+        <f>'Jan 2026 A vs F '!B9</f>
         <v>144779.5</v>
       </c>
       <c r="D8" s="100">
-        <f>'Jan 2026 A vs F '!C8</f>
+        <f>'Jan 2026 A vs F '!C9</f>
         <v>146831.05083333334</v>
       </c>
       <c r="E8" s="100">
-        <f>'Jan 2026 A vs F '!D8</f>
+        <f>'Jan 2026 A vs F '!D9</f>
         <v>-2051.5508333333419</v>
       </c>
     </row>
@@ -19552,35 +19579,35 @@
       </c>
     </row>
     <row r="34" spans="1:27" ht="80" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A34" s="113" t="s">
+      <c r="A34" s="127" t="s">
         <v>188</v>
       </c>
-      <c r="B34" s="114"/>
-      <c r="C34" s="114"/>
-      <c r="D34" s="114"/>
-      <c r="E34" s="114"/>
-      <c r="F34" s="114"/>
-      <c r="G34" s="114"/>
-      <c r="H34" s="114"/>
-      <c r="I34" s="114"/>
-      <c r="J34" s="114"/>
-      <c r="K34" s="114"/>
-      <c r="L34" s="114"/>
-      <c r="M34" s="114"/>
-      <c r="N34" s="114"/>
-      <c r="O34" s="114"/>
-      <c r="P34" s="114"/>
-      <c r="Q34" s="114"/>
-      <c r="R34" s="114"/>
-      <c r="S34" s="114"/>
-      <c r="T34" s="114"/>
-      <c r="U34" s="114"/>
-      <c r="V34" s="114"/>
-      <c r="W34" s="114"/>
-      <c r="X34" s="114"/>
-      <c r="Y34" s="114"/>
-      <c r="Z34" s="114"/>
-      <c r="AA34" s="114"/>
+      <c r="B34" s="128"/>
+      <c r="C34" s="128"/>
+      <c r="D34" s="128"/>
+      <c r="E34" s="128"/>
+      <c r="F34" s="128"/>
+      <c r="G34" s="128"/>
+      <c r="H34" s="128"/>
+      <c r="I34" s="128"/>
+      <c r="J34" s="128"/>
+      <c r="K34" s="128"/>
+      <c r="L34" s="128"/>
+      <c r="M34" s="128"/>
+      <c r="N34" s="128"/>
+      <c r="O34" s="128"/>
+      <c r="P34" s="128"/>
+      <c r="Q34" s="128"/>
+      <c r="R34" s="128"/>
+      <c r="S34" s="128"/>
+      <c r="T34" s="128"/>
+      <c r="U34" s="128"/>
+      <c r="V34" s="128"/>
+      <c r="W34" s="128"/>
+      <c r="X34" s="128"/>
+      <c r="Y34" s="128"/>
+      <c r="Z34" s="128"/>
+      <c r="AA34" s="128"/>
     </row>
     <row r="35" spans="1:27" ht="15" customHeight="1" x14ac:dyDescent="0.35"/>
     <row r="36" spans="1:27" x14ac:dyDescent="0.35">
@@ -19589,35 +19616,35 @@
       </c>
     </row>
     <row r="37" spans="1:27" ht="95" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A37" s="113" t="s">
+      <c r="A37" s="127" t="s">
         <v>190</v>
       </c>
-      <c r="B37" s="114"/>
-      <c r="C37" s="114"/>
-      <c r="D37" s="114"/>
-      <c r="E37" s="114"/>
-      <c r="F37" s="114"/>
-      <c r="G37" s="114"/>
-      <c r="H37" s="114"/>
-      <c r="I37" s="114"/>
-      <c r="J37" s="114"/>
-      <c r="K37" s="114"/>
-      <c r="L37" s="114"/>
-      <c r="M37" s="114"/>
-      <c r="N37" s="114"/>
-      <c r="O37" s="114"/>
-      <c r="P37" s="114"/>
-      <c r="Q37" s="114"/>
-      <c r="R37" s="114"/>
-      <c r="S37" s="114"/>
-      <c r="T37" s="114"/>
-      <c r="U37" s="114"/>
-      <c r="V37" s="114"/>
-      <c r="W37" s="114"/>
-      <c r="X37" s="114"/>
-      <c r="Y37" s="114"/>
-      <c r="Z37" s="114"/>
-      <c r="AA37" s="114"/>
+      <c r="B37" s="128"/>
+      <c r="C37" s="128"/>
+      <c r="D37" s="128"/>
+      <c r="E37" s="128"/>
+      <c r="F37" s="128"/>
+      <c r="G37" s="128"/>
+      <c r="H37" s="128"/>
+      <c r="I37" s="128"/>
+      <c r="J37" s="128"/>
+      <c r="K37" s="128"/>
+      <c r="L37" s="128"/>
+      <c r="M37" s="128"/>
+      <c r="N37" s="128"/>
+      <c r="O37" s="128"/>
+      <c r="P37" s="128"/>
+      <c r="Q37" s="128"/>
+      <c r="R37" s="128"/>
+      <c r="S37" s="128"/>
+      <c r="T37" s="128"/>
+      <c r="U37" s="128"/>
+      <c r="V37" s="128"/>
+      <c r="W37" s="128"/>
+      <c r="X37" s="128"/>
+      <c r="Y37" s="128"/>
+      <c r="Z37" s="128"/>
+      <c r="AA37" s="128"/>
     </row>
   </sheetData>
   <mergeCells count="2">

</xml_diff>